<commit_message>
Added SESTDTC and ETCD to output variables.
</commit_message>
<xml_diff>
--- a/rules/CORE-000527/negative/01/data/unit-test-coreid-CG0209-negative.xlsx
+++ b/rules/CORE-000527/negative/01/data/unit-test-coreid-CG0209-negative.xlsx
@@ -53,11 +53,11 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -87,6 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -121,8 +122,8 @@
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -467,10 +468,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -494,10 +495,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Subject Elements</v>
       </c>
     </row>
@@ -510,7 +511,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -546,12 +547,52 @@
         <v>16</v>
       </c>
       <c r="E2" s="2" t="str">
+        <v>ETCD</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="str">
+        <v>se.xpt</v>
+      </c>
+      <c r="C3" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="4">
+        <v>16</v>
+      </c>
+      <c r="E3" s="4" t="str">
         <v>SEENDTC</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>se.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>SESTDTC</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>2013-02-19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -596,515 +637,515 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="5" t="str">
         <v>Element Code</v>
       </c>
-      <c r="F2" s="4" t="str">
+      <c r="F2" s="5" t="str">
         <v>Description of Element</v>
       </c>
-      <c r="G2" s="4" t="str">
+      <c r="G2" s="5" t="str">
         <v>Epoch</v>
       </c>
-      <c r="H2" s="4" t="str">
+      <c r="H2" s="5" t="str">
         <v>Start Date/Time of Element</v>
       </c>
-      <c r="I2" s="4" t="str">
+      <c r="I2" s="5" t="str">
         <v>End Date/Time of Element</v>
       </c>
-      <c r="J2" s="4" t="str">
+      <c r="J2" s="5" t="str">
         <v>Study Day of Start of Element</v>
       </c>
-      <c r="K2" s="4" t="str">
+      <c r="K2" s="5" t="str">
         <v>Study Day of End of Element</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="4" t="str">
+      <c r="G3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="H3" s="4" t="str">
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="4" t="str">
+      <c r="I3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="4" t="str">
+      <c r="J3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="K3" s="4" t="str">
+      <c r="K3" s="5" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="5">
         <v>7</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="5">
         <v>26</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="5">
         <v>9</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="5">
         <v>10</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="5">
         <v>10</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="5">
         <v>8</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="5">
         <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C5" s="5" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="5">
-        <v>1</v>
-      </c>
-      <c r="E5" s="5" t="str">
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="str">
         <v>SCREEN</v>
       </c>
-      <c r="F5" s="5" t="str">
+      <c r="F5" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G5" s="5" t="str">
+      <c r="G5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H5" s="4" t="str">
         <v>2012-11-23</v>
       </c>
-      <c r="I5" s="5" t="str">
+      <c r="I5" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="4">
         <v>-7</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>LOW</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>Zanomaline 54 mg</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H6" s="6" t="str">
+      <c r="H6" s="4" t="str">
         <v>2012-11-30</v>
       </c>
-      <c r="I6" s="6" t="str">
+      <c r="I6" s="4" t="str">
         <v>2013-05-20</v>
       </c>
-      <c r="J6" s="6">
-        <v>1</v>
-      </c>
-      <c r="K6" s="6">
+      <c r="J6" s="4">
+        <v>1</v>
+      </c>
+      <c r="K6" s="4">
         <v>172</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="5" t="str">
+      <c r="B7" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C7" s="5" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D7" s="5">
-        <v>1</v>
-      </c>
-      <c r="E7" s="5" t="str">
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="str">
         <v>SCREEN</v>
       </c>
-      <c r="F7" s="5" t="str">
+      <c r="F7" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G7" s="5" t="str">
+      <c r="G7" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H7" s="5" t="str">
+      <c r="H7" s="4" t="str">
         <v>2012-10-30</v>
       </c>
-      <c r="I7" s="5" t="str">
+      <c r="I7" s="4" t="str">
         <v>2012-11-15</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="4">
         <v>-16</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
         <v>2</v>
       </c>
-      <c r="E8" s="6" t="str">
+      <c r="E8" s="4" t="str">
         <v>LOW</v>
       </c>
-      <c r="F8" s="6" t="str">
+      <c r="F8" s="4" t="str">
         <v>Zanomaline 54 mg</v>
       </c>
-      <c r="G8" s="6" t="str">
+      <c r="G8" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H8" s="6" t="str">
+      <c r="H8" s="4" t="str">
         <v>2012-11-15</v>
       </c>
-      <c r="I8" s="6" t="str">
+      <c r="I8" s="4" t="str">
         <v>2013-01-14</v>
       </c>
-      <c r="J8" s="6">
-        <v>1</v>
-      </c>
-      <c r="K8" s="6">
+      <c r="J8" s="4">
+        <v>1</v>
+      </c>
+      <c r="K8" s="4">
         <v>61</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="str">
+      <c r="A9" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B9" s="5" t="str">
+      <c r="B9" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C9" s="5" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D9" s="5">
-        <v>1</v>
-      </c>
-      <c r="E9" s="5" t="str">
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="str">
         <v>SCREEN</v>
       </c>
-      <c r="F9" s="5" t="str">
+      <c r="F9" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G9" s="5" t="str">
+      <c r="G9" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H9" s="5" t="str">
+      <c r="H9" s="4" t="str">
         <v>2013-08-20</v>
       </c>
-      <c r="I9" s="5" t="str">
+      <c r="I9" s="4" t="str">
         <v>2013-08-29</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="4">
         <v>-9</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="str">
+      <c r="A10" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B10" s="6" t="str">
+      <c r="B10" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="4">
         <v>2</v>
       </c>
-      <c r="E10" s="6" t="str">
+      <c r="E10" s="4" t="str">
         <v>TITRATE</v>
       </c>
-      <c r="F10" s="6" t="str">
+      <c r="F10" s="4" t="str">
         <v>Zanomaline 54 mg Titration</v>
       </c>
-      <c r="G10" s="6" t="str">
+      <c r="G10" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H10" s="6" t="str">
+      <c r="H10" s="4" t="str">
         <v>2013-08-29</v>
       </c>
-      <c r="I10" s="6" t="str">
+      <c r="I10" s="4" t="str">
         <v>2013-09-15</v>
       </c>
-      <c r="J10" s="6">
-        <v>1</v>
-      </c>
-      <c r="K10" s="6">
+      <c r="J10" s="4">
+        <v>1</v>
+      </c>
+      <c r="K10" s="4">
         <v>18</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="str">
+      <c r="A11" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B11" s="5" t="str">
+      <c r="B11" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C11" s="5" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>3</v>
       </c>
-      <c r="E11" s="5" t="str">
+      <c r="E11" s="4" t="str">
         <v>HIGH</v>
       </c>
-      <c r="F11" s="5" t="str">
+      <c r="F11" s="4" t="str">
         <v>Zanomaline 81 mg</v>
       </c>
-      <c r="G11" s="5" t="str">
+      <c r="G11" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H11" s="5" t="str">
+      <c r="H11" s="4" t="str">
         <v>2013-09-15</v>
       </c>
-      <c r="I11" s="5" t="str">
+      <c r="I11" s="4" t="str">
         <v/>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="4">
         <v>18</v>
       </c>
-      <c r="K11" s="5" t="str">
+      <c r="K11" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="str">
+      <c r="A12" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B12" s="6" t="str">
+      <c r="B12" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C12" s="6" t="str">
+      <c r="C12" s="4" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D12" s="6">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6" t="str">
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="str">
         <v>SCREEN</v>
       </c>
-      <c r="F12" s="6" t="str">
+      <c r="F12" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G12" s="6" t="str">
+      <c r="G12" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H12" s="6" t="str">
+      <c r="H12" s="4" t="str">
         <v>2013-10-01</v>
       </c>
-      <c r="I12" s="6" t="str">
+      <c r="I12" s="4" t="str">
         <v>2013-10-08</v>
       </c>
-      <c r="J12" s="6">
+      <c r="J12" s="4">
         <v>-7</v>
       </c>
-      <c r="K12" s="6">
+      <c r="K12" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="str">
+      <c r="A13" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B13" s="5" t="str">
+      <c r="B13" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C13" s="5" t="str">
+      <c r="C13" s="4" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>2</v>
       </c>
-      <c r="E13" s="5" t="str">
+      <c r="E13" s="4" t="str">
         <v>PLACEBO</v>
       </c>
-      <c r="F13" s="5" t="str">
+      <c r="F13" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="G13" s="5" t="str">
+      <c r="G13" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H13" s="5" t="str">
+      <c r="H13" s="4" t="str">
         <v>2013-10-08</v>
       </c>
-      <c r="I13" s="5" t="str">
+      <c r="I13" s="4" t="str">
         <v>2014-03-18</v>
       </c>
-      <c r="J13" s="5">
-        <v>1</v>
-      </c>
-      <c r="K13" s="5">
+      <c r="J13" s="4">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4">
         <v>162</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="str">
+      <c r="A14" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B14" s="6" t="str">
+      <c r="B14" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C14" s="6" t="str">
+      <c r="C14" s="4" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D14" s="6">
-        <v>1</v>
-      </c>
-      <c r="E14" s="6" t="str">
+      <c r="D14" s="4">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="str">
         <v>SCREEN</v>
       </c>
-      <c r="F14" s="6" t="str">
+      <c r="F14" s="4" t="str">
         <v>Screening</v>
       </c>
-      <c r="G14" s="6" t="str">
+      <c r="G14" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H14" s="6" t="str">
+      <c r="H14" s="4" t="str">
         <v>2013-01-22</v>
       </c>
-      <c r="I14" s="6" t="str">
+      <c r="I14" s="4" t="str">
         <v>2013-02-04</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J14" s="4">
         <v>-13</v>
       </c>
-      <c r="K14" s="6">
+      <c r="K14" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="str">
+      <c r="A15" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B15" s="5" t="str">
+      <c r="B15" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C15" s="5" t="str">
+      <c r="C15" s="4" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <v>2</v>
       </c>
-      <c r="E15" s="5" t="str">
+      <c r="E15" s="4" t="str">
         <v>TITRATE</v>
       </c>
-      <c r="F15" s="5" t="str">
+      <c r="F15" s="4" t="str">
         <v>Zanomaline 54 mg Titration</v>
       </c>
-      <c r="G15" s="5" t="str">
+      <c r="G15" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H15" s="5" t="str">
+      <c r="H15" s="4" t="str">
         <v>2013-02-04</v>
       </c>
-      <c r="I15" s="5" t="str">
+      <c r="I15" s="4" t="str">
         <v>2013-02-19</v>
       </c>
-      <c r="J15" s="5">
-        <v>1</v>
-      </c>
-      <c r="K15" s="5">
+      <c r="J15" s="4">
+        <v>1</v>
+      </c>
+      <c r="K15" s="4">
         <v>16</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="str">
+      <c r="A16" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B16" s="6" t="str">
+      <c r="B16" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C16" s="6" t="str">
+      <c r="C16" s="4" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="4">
         <v>3</v>
       </c>
       <c r="E16" s="6" t="str">
         <v>HIGH</v>
       </c>
-      <c r="F16" s="6" t="str">
+      <c r="F16" s="4" t="str">
         <v>Zanomaline 81 mg</v>
       </c>
-      <c r="G16" s="6" t="str">
+      <c r="G16" s="4" t="str">
         <v>TREATMENT</v>
       </c>
       <c r="H16" s="6" t="str">
@@ -1113,45 +1154,45 @@
       <c r="I16" s="7" t="str">
         <v/>
       </c>
-      <c r="J16" s="6">
+      <c r="J16" s="4">
         <v>16</v>
       </c>
-      <c r="K16" s="6" t="str">
+      <c r="K16" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="str">
+      <c r="A17" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B17" s="5" t="str">
+      <c r="B17" s="4" t="str">
         <v>SE</v>
       </c>
-      <c r="C17" s="5" t="str">
+      <c r="C17" s="4" t="str">
         <v>CDISC005</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <v>4</v>
       </c>
-      <c r="E17" s="5" t="str">
+      <c r="E17" s="4" t="str">
         <v>TITRATE</v>
       </c>
-      <c r="F17" s="5" t="str">
+      <c r="F17" s="4" t="str">
         <v>Zanomaline 54 mg Titration</v>
       </c>
-      <c r="G17" s="5" t="str">
+      <c r="G17" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H17" s="5" t="str">
+      <c r="H17" s="4" t="str">
         <v>2013-07-30</v>
       </c>
-      <c r="I17" s="5" t="str">
+      <c r="I17" s="4" t="str">
         <v>2013-08-06</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="4">
         <v>177</v>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="4">
         <v>184</v>
       </c>
     </row>

</xml_diff>